<commit_message>
Give the SLA chart the red line its caption promises
"Area past the red line is a breach" was drawn with a line series holding one
point and no marker. A category chart takes one Y per X, so an X-axis limit can
only ever be a single point, and a single point with no marker draws nothing —
Excel and LibreOffice both agree. The caption named a line that was not there.

A one-category column with a wide gap is a vertical rule, and it is the only
shape on a category chart that is, so _vrule() adds one as a combo sub-chart.

Also: a horizontal chart's last value label is centred on the end of the axis,
so half of it hung past the plot and the DPMO scale read "400,00(".
</commit_message>
<xml_diff>
--- a/templates/19-black-belt-calculators.xlsx
+++ b/templates/19-black-belt-calculators.xlsx
@@ -1062,6 +1062,12 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="1"/>
           <order val="1"/>
@@ -1069,36 +1075,26 @@
             <v>SLA limit</v>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:solidFill>
+              <a:srgbClr val="C0392B"/>
+            </a:solidFill>
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="C0392B"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'3 SLA capability'!$A$21:$A$61</f>
-            </numRef>
-          </cat>
           <val>
             <numRef>
               <f>'3 SLA capability'!$C$21:$C$61</f>
             </numRef>
           </val>
-          <smooth val="0"/>
         </ser>
+        <gapWidth val="400"/>
         <axId val="10"/>
         <axId val="100"/>
-      </lineChart>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>

</xml_diff>